<commit_message>
Add new validations. file view option to admin
</commit_message>
<xml_diff>
--- a/Documents/Copy of Sub-lang-country-TV-2026-Translation Document TR.xlsx
+++ b/Documents/Copy of Sub-lang-country-TV-2026-Translation Document TR.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CRM 2.0\Adobe Web Forms\TV2H26\Subsidairy\SETK\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Adobe-Form-Builder-main\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7284A326-4E00-43A2-9E43-7887D1E17DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB75DDEE-3B79-4CE0-B897-639C203DC8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29280" yWindow="2310" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1710" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TV-2026 Translations" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="191">
   <si>
     <t>Translation</t>
   </si>
@@ -605,6 +605,12 @@
   </si>
   <si>
     <t>(Tek yanıt)</t>
+  </si>
+  <si>
+    <t>TV2H26</t>
+  </si>
+  <si>
+    <t>Project Code</t>
   </si>
 </sst>
 </file>
@@ -1089,8 +1095,12 @@
     </row>
     <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16"/>
-      <c r="B2"/>
-      <c r="C2" s="17"/>
+      <c r="B2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>189</v>
+      </c>
       <c r="D2" s="17"/>
     </row>
     <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>